<commit_message>
State that neither ultrasound reader reported an audited examination
The authors confirmed that neither of the two readers who coded the
ultrasound report content (the ultrasound physician and the pediatric
surgeon, both authors) issued any of the audited ultrasound reports. The
Methods, the Table 3 note and Supplement 1 (K3) now say so. To make room
under the word limit, "that other departments can apply" is cut from the
last paragraph of the Introduction, where the Discussion and the Take-Home
Points already say it.

Main text 2,998 words, abstract 249. jacr_check passes; verify_numbers.py:
311 rows, 265 consistent, 46 definitional, 0 inconsistent.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TkounLTBFVQRstE3VnhkM
</commit_message>
<xml_diff>
--- a/数字核对表.xlsx
+++ b/数字核对表.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">专项检查!$A$1:$B$8</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">更正记录!$A$1:$D$30</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">更正记录!$A$1:$D$31</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$312</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">问题汇总!$A$1:$F$1</definedName>
   </definedNames>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1725" uniqueCount="962">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1729" uniqueCount="966">
   <si>
     <r>
       <rPr>
@@ -31328,7 +31328,7 @@
     <t xml:space="preserve">Title Page · Word count</t>
   </si>
   <si>
-    <t xml:space="preserve">2,996 … Abstract: 249 words</t>
+    <t xml:space="preserve">2,998 … Abstract: 249 words</t>
   </si>
   <si>
     <r>
@@ -31363,7 +31363,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2996</t>
+      <t xml:space="preserve">2998</t>
     </r>
     <r>
       <rPr>
@@ -31486,7 +31486,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Word count: 2,996 … Tables: 4; Figures: 3; Supplements 1–4</t>
+    <t xml:space="preserve">Word count: 2,998 … Tables: 4; Figures: 3; Supplements 1–4</t>
   </si>
   <si>
     <r>
@@ -31504,7 +31504,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2996</t>
+      <t xml:space="preserve">2998</t>
     </r>
   </si>
   <si>
@@ -37911,6 +37911,109 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">n</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">方法 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">内容编码；表 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">注；补充</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 · K3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（阅读者与报告）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">both authors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">both authors who had reported none of the examinations</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用户 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">确认两位超声阅读者均未出具被审计的超声报告；为腾字数删去引言末段 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"that other departments can apply"</t>
     </r>
   </si>
   <si>
@@ -44264,7 +44367,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -44678,22 +44781,36 @@
         <v>957</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
         <v>958</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>959</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="9" t="s">
         <v>960</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="8" t="s">
         <v>961</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>962</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>963</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>964</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>965</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D30"/>
+  <autoFilter ref="A1:D31"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Polish the English of the manuscript text
Shorter sentences, fewer repeated clauses and more standard phrasing in the
abstract, Introduction, Methods, Results, Discussion, Limitations, Take-Home
Points, supplement list and figure legends. Numbers, number words, reference
numbers and abbreviations are unchanged, as is the statistical analysis paragraph
and the Declarations. Main text 2,976 words; number check 354 rows, 0 inconsistent.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TkounLTBFVQRstE3VnhkM
</commit_message>
<xml_diff>
--- a/数字核对表.xlsx
+++ b/数字核对表.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">专项检查!$A$1:$B$8</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">更正记录!$A$1:$D$34</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$356</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$355</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">问题汇总!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="1085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1956" uniqueCount="1083">
   <si>
     <r>
       <rPr>
@@ -35340,7 +35340,7 @@
     <t xml:space="preserve">Title Page · Word count</t>
   </si>
   <si>
-    <t xml:space="preserve">2,996 … Abstract: 248 words</t>
+    <t xml:space="preserve">2,976 … Abstract: 248 words</t>
   </si>
   <si>
     <r>
@@ -35375,7 +35375,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2996</t>
+      <t xml:space="preserve">2976</t>
     </r>
     <r>
       <rPr>
@@ -35498,7 +35498,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Word count: 2,996 … Tables: 4; Figures: 3; Supplements 1–4</t>
+    <t xml:space="preserve">Word count: 2,976 … Tables: 4; Figures: 3; Supplements 1–4</t>
   </si>
   <si>
     <r>
@@ -35516,7 +35516,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2996</t>
+      <t xml:space="preserve">2976</t>
     </r>
   </si>
   <si>
@@ -37162,7 +37162,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">three of</t>
+      <t xml:space="preserve">three as</t>
     </r>
     <r>
       <rPr>
@@ -37832,61 +37832,6 @@
   </si>
   <si>
     <t xml:space="preserve">all three examinations</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">图注 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· Figure 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（计数词）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> one of</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">；</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">one of the three index</t>
-    </r>
   </si>
   <si>
     <r>
@@ -45213,7 +45158,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">COUNTA(核对表!B2:B2000)</f>
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45258,7 +45203,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTIF(核对表!C2:C2000,"【定义/描述性数字】*")</f>
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45286,7 +45231,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E355"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -51297,7 +51242,7 @@
       </c>
     </row>
     <row r="354" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A354" s="10" t="s">
+      <c r="A354" s="11" t="s">
         <v>944</v>
       </c>
       <c r="B354" s="11" t="s">
@@ -51330,25 +51275,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="356" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A356" s="11" t="s">
-        <v>948</v>
-      </c>
-      <c r="B356" s="11" t="s">
-        <v>949</v>
-      </c>
-      <c r="C356" s="10" t="s">
-        <v>893</v>
-      </c>
-      <c r="D356" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E356" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E356"/>
+  <autoFilter ref="A1:E355"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -51377,7 +51305,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>23</v>
@@ -51422,66 +51350,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
     </row>
   </sheetData>
@@ -51515,27 +51443,27 @@
         <v>23</v>
       </c>
       <c r="B1" s="7" t="s">
+        <v>965</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>966</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>967</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>968</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
+        <v>968</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>969</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>970</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>971</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>972</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>973</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51543,13 +51471,13 @@
         <v>38</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>972</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>973</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>974</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>975</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>976</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51557,13 +51485,13 @@
         <v>134</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>975</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>976</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>977</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>978</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>979</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51571,13 +51499,13 @@
         <v>277</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>978</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>979</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>980</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>981</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>982</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51585,27 +51513,27 @@
         <v>283</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
+        <v>983</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>984</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>985</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>986</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>987</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>988</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51613,27 +51541,27 @@
         <v>111</v>
       </c>
       <c r="B8" s="9" t="s">
+        <v>987</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>988</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>989</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>990</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>991</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>69</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51641,13 +51569,13 @@
         <v>127</v>
       </c>
       <c r="B10" s="9" t="s">
+        <v>993</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>994</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>995</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>996</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51655,13 +51583,13 @@
         <v>146</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>996</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>997</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>998</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>999</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>1000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51669,13 +51597,13 @@
         <v>368</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>999</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>1001</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>1002</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>1003</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51683,13 +51611,13 @@
         <v>382</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>1004</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>1005</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>1006</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51697,13 +51625,13 @@
         <v>385</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>1006</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>1007</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>1008</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>1009</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51711,13 +51639,13 @@
         <v>397</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>1010</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>1011</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>1012</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51725,265 +51653,265 @@
         <v>406</v>
       </c>
       <c r="B16" s="9" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>1012</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>1013</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>1014</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>1015</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>1016</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="D17" s="9" t="s">
         <v>1017</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>1018</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>1020</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="D18" s="8" t="s">
         <v>1021</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>1022</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>1023</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>1024</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>1025</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>1026</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>1027</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>1028</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="D20" s="8" t="s">
         <v>1029</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>1030</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>1031</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>1032</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="D21" s="8" t="s">
         <v>1033</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>1034</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>1035</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>1036</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="D22" s="8" t="s">
         <v>1037</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>1038</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>1039</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>1040</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="D23" s="8" t="s">
         <v>1041</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>1042</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>1043</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>1044</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="D24" s="8" t="s">
         <v>1045</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>1046</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>1047</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>1048</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>1049</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>1038</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>1050</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>1054</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="D27" s="8" t="s">
         <v>1055</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>1056</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>1057</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>1060</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>1061</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="D29" s="8" t="s">
         <v>1062</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>1063</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C30" s="9" t="s">
         <v>1065</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="D30" s="8" t="s">
         <v>1066</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>1067</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>1068</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C31" s="9" t="s">
         <v>1069</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="D31" s="8" t="s">
         <v>1070</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>1071</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>1072</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>1073</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="D32" s="9" t="s">
         <v>1074</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>1075</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>1076</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="69.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C33" s="9" t="s">
         <v>1077</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="D33" s="8" t="s">
         <v>1078</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>1079</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>1080</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>1081</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="D34" s="9" t="s">
         <v>1082</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>1083</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>1084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final pre-submission fixes to the submission package
Code spans render in monospace instead of showing backticks. Tables are cited in
order in the Methods. Supplement 2 no longer refers to a non-existent S2.10.
Supplementary tables are renumbered S1-S19 in the order they appear, and the
subtitles of Supplements 3 and 4 name the paper. The Discussion calls the
published figures sensitivities. Supplement 3 no longer states untested
explanations for CT detection. Figure 1 and Figure 3A labels are corrected.
The cover letter is dated October 10, 2026 and the operations sheet matches the
manuscript.

Main text 2,978 words; number check 355 rows, 0 inconsistent; JACR checks pass.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TkounLTBFVQRstE3VnhkM
</commit_message>
<xml_diff>
--- a/数字核对表.xlsx
+++ b/数字核对表.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">专项检查!$A$1:$B$8</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">更正记录!$A$1:$D$34</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$355</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$356</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">问题汇总!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1956" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1961" uniqueCount="1085">
   <si>
     <r>
       <rPr>
@@ -167,7 +167,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S1–S15</t>
+      <t xml:space="preserve">S1–S19</t>
     </r>
     <r>
       <rPr>
@@ -4715,7 +4715,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9 </t>
+      <t xml:space="preserve">S8 </t>
     </r>
     <r>
       <rPr>
@@ -19593,7 +19593,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S10</t>
+      <t xml:space="preserve">S9</t>
     </r>
     <r>
       <rPr>
@@ -20719,7 +20719,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Third portion of the duodenum (D3)</t>
+      <t xml:space="preserve">S19 · Third portion of the duodenum (D3)</t>
     </r>
   </si>
   <si>
@@ -20836,7 +20836,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Duodenojejunal junction</t>
+      <t xml:space="preserve">S19 · Duodenojejunal junction</t>
     </r>
   </si>
   <si>
@@ -20953,7 +20953,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Superior mesenteric artery–vein relationship</t>
+      <t xml:space="preserve">S19 · Superior mesenteric artery–vein relationship</t>
     </r>
   </si>
   <si>
@@ -21033,7 +21033,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Enteric fluid</t>
+      <t xml:space="preserve">S19 · Enteric fluid</t>
     </r>
   </si>
   <si>
@@ -21116,7 +21116,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Dynamic assessment</t>
+      <t xml:space="preserve">S19 · Dynamic assessment</t>
     </r>
   </si>
   <si>
@@ -21199,7 +21199,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Graded compression</t>
+      <t xml:space="preserve">S19 · Graded compression</t>
     </r>
   </si>
   <si>
@@ -21279,7 +21279,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Color Doppler of the mesenteric vessels</t>
+      <t xml:space="preserve">S19 · Color Doppler of the mesenteric vessels</t>
     </r>
   </si>
   <si>
@@ -21362,7 +21362,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Whirlpool sign</t>
+      <t xml:space="preserve">S19 · Whirlpool sign</t>
     </r>
   </si>
   <si>
@@ -21445,7 +21445,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Study adequacy</t>
+      <t xml:space="preserve">S19 · Study adequacy</t>
     </r>
   </si>
   <si>
@@ -21528,7 +21528,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Duodenum mentioned in any form</t>
+      <t xml:space="preserve">S19 · Duodenum mentioned in any form</t>
     </r>
   </si>
   <si>
@@ -21611,7 +21611,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Explicit statement of vessel inversion</t>
+      <t xml:space="preserve">S19 · Explicit statement of vessel inversion</t>
     </r>
   </si>
   <si>
@@ -21647,7 +21647,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 · Cecal position</t>
+      <t xml:space="preserve">S19 · Cecal position</t>
     </r>
   </si>
   <si>
@@ -26962,7 +26962,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Contrast enhancement</t>
+      <t xml:space="preserve">S18 · Contrast enhancement</t>
     </r>
   </si>
   <si>
@@ -27096,7 +27096,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Mesenteric whirl</t>
+      <t xml:space="preserve">S18 · Mesenteric whirl</t>
     </r>
   </si>
   <si>
@@ -27230,7 +27230,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Duodenum mentioned</t>
+      <t xml:space="preserve">S18 · Duodenum mentioned</t>
     </r>
   </si>
   <si>
@@ -27364,7 +27364,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Mesenteric-vessel relationship</t>
+      <t xml:space="preserve">S18 · Mesenteric-vessel relationship</t>
     </r>
   </si>
   <si>
@@ -27498,7 +27498,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Three-dimensional reconstruction</t>
+      <t xml:space="preserve">S18 · Three-dimensional reconstruction</t>
     </r>
   </si>
   <si>
@@ -27632,7 +27632,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Duodenojejunal junction</t>
+      <t xml:space="preserve">S18 · Duodenojejunal junction</t>
     </r>
   </si>
   <si>
@@ -27766,7 +27766,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Corkscrew / spring appearance</t>
+      <t xml:space="preserve">S18 · Corkscrew / spring appearance</t>
     </r>
   </si>
   <si>
@@ -27900,7 +27900,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Jejunal position</t>
+      <t xml:space="preserve">S18 · Jejunal position</t>
     </r>
   </si>
   <si>
@@ -28034,7 +28034,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Cecal position</t>
+      <t xml:space="preserve">S18 · Cecal position</t>
     </r>
   </si>
   <si>
@@ -28168,7 +28168,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Whole-gastrointestinal study</t>
+      <t xml:space="preserve">S18 · Whole-gastrointestinal study</t>
     </r>
   </si>
   <si>
@@ -28302,7 +28302,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 · Barium used</t>
+      <t xml:space="preserve">S18 · Barium used</t>
     </r>
   </si>
   <si>
@@ -28436,7 +28436,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9 · </t>
+      <t xml:space="preserve">S8 · </t>
     </r>
     <r>
       <rPr>
@@ -28621,7 +28621,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9 · </t>
+      <t xml:space="preserve">S8 · </t>
     </r>
     <r>
       <rPr>
@@ -28806,7 +28806,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9 · </t>
+      <t xml:space="preserve">S8 · </t>
     </r>
     <r>
       <rPr>
@@ -28991,7 +28991,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9 · </t>
+      <t xml:space="preserve">S8 · </t>
     </r>
     <r>
       <rPr>
@@ -29176,7 +29176,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S10 · D3 or duodenojejunal junction</t>
+      <t xml:space="preserve">S9 · D3 or duodenojejunal junction</t>
     </r>
   </si>
   <si>
@@ -29327,7 +29327,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S10 · Superior mesenteric artery–vein relationship</t>
+      <t xml:space="preserve">S9 · Superior mesenteric artery–vein relationship</t>
     </r>
   </si>
   <si>
@@ -29363,7 +29363,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S10 · Enteric fluid administration</t>
+      <t xml:space="preserve">S9 · Enteric fluid administration</t>
     </r>
   </si>
   <si>
@@ -29514,7 +29514,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S10 · Whirlpool, swirl or spiral appearance reported</t>
+      <t xml:space="preserve">S9 · Whirlpool, swirl or spiral appearance reported</t>
     </r>
   </si>
   <si>
@@ -29665,7 +29665,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S11 · Explicit operative statement of torsion,</t>
+      <t xml:space="preserve">S10 · Explicit operative statement of torsion,</t>
     </r>
   </si>
   <si>
@@ -29765,7 +29765,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S11 · Excluding children whose record states a</t>
+      <t xml:space="preserve">S10 · Excluding children whose record states a</t>
     </r>
   </si>
   <si>
@@ -29865,7 +29865,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S11 · Requiring a documented rotation of 360° </t>
+      <t xml:space="preserve">S10 · Requiring a documented rotation of 360° </t>
     </r>
   </si>
   <si>
@@ -29965,7 +29965,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S12 · Ultrasound, crude</t>
+      <t xml:space="preserve">S11 · Ultrasound, crude</t>
     </r>
   </si>
   <si>
@@ -30099,7 +30099,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S12 · Ultrasound, adjusted for great-vessel session</t>
+      <t xml:space="preserve">S11 · Ultrasound, adjusted for great-vessel session</t>
     </r>
   </si>
   <si>
@@ -30233,7 +30233,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S12 · CT, crude</t>
+      <t xml:space="preserve">S11 · CT, crude</t>
     </r>
   </si>
   <si>
@@ -30367,7 +30367,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S12 · CT, adjusted for contrast enhancement</t>
+      <t xml:space="preserve">S11 · CT, adjusted for contrast enhancement</t>
     </r>
   </si>
   <si>
@@ -30501,7 +30501,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S12 · UGI series, crude</t>
+      <t xml:space="preserve">S11 · UGI series, crude</t>
     </r>
   </si>
   <si>
@@ -30635,7 +30635,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S13 · UGI series vs CT</t>
+      <t xml:space="preserve">S12 · UGI series vs CT</t>
     </r>
   </si>
   <si>
@@ -30752,7 +30752,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S13 · UGI series vs ultrasound</t>
+      <t xml:space="preserve">S12 · UGI series vs ultrasound</t>
     </r>
   </si>
   <si>
@@ -30869,7 +30869,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S13 · CT vs ultrasound</t>
+      <t xml:space="preserve">S12 · CT vs ultrasound</t>
     </r>
   </si>
   <si>
@@ -30986,7 +30986,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S14 · UGI vs CT × </t>
+      <t xml:space="preserve">S13 · UGI vs CT × </t>
     </r>
     <r>
       <rPr>
@@ -31094,7 +31094,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S14 · </t>
+      <t xml:space="preserve">S13 · </t>
     </r>
     <r>
       <rPr>
@@ -31202,7 +31202,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S14 · Firth</t>
+      <t xml:space="preserve">S13 · Firth</t>
     </r>
   </si>
   <si>
@@ -31302,7 +31302,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S14 · </t>
+      <t xml:space="preserve">S13 · </t>
     </r>
     <r>
       <rPr>
@@ -31461,7 +31461,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S14 · CT </t>
+      <t xml:space="preserve">S13 · CT </t>
     </r>
     <r>
       <rPr>
@@ -31787,7 +31787,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S16 · Primary: final label</t>
+      <t xml:space="preserve">S14 · Primary: final label</t>
     </r>
   </si>
   <si>
@@ -31972,7 +31972,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S16 · Conclusion names malrotation</t>
+      <t xml:space="preserve">S14 · Conclusion names malrotation</t>
     </r>
   </si>
   <si>
@@ -32157,7 +32157,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S16 · Possible-tier conclusions counted negative</t>
+      <t xml:space="preserve">S14 · Possible-tier conclusions counted negative</t>
     </r>
   </si>
   <si>
@@ -32342,7 +32342,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S16 · Conclusion-only classifier (Supplement_1_classifier.py)</t>
+      <t xml:space="preserve">S14 · Conclusion-only classifier (Supplement_1_classifier.py)</t>
     </r>
   </si>
   <si>
@@ -32527,7 +32527,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S17 · Primary: final label</t>
+      <t xml:space="preserve">S15 · Primary: final label</t>
     </r>
   </si>
   <si>
@@ -32763,7 +32763,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S17 · Conclusion names malrotation</t>
+      <t xml:space="preserve">S15 · Conclusion names malrotation</t>
     </r>
   </si>
   <si>
@@ -32948,7 +32948,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S17 · Possible-tier conclusions counted negative</t>
+      <t xml:space="preserve">S15 · Possible-tier conclusions counted negative</t>
     </r>
   </si>
   <si>
@@ -33133,7 +33133,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S17 · Conclusion-only classifier (Supplement_1_classifier.py)</t>
+      <t xml:space="preserve">S15 · Conclusion-only classifier (Supplement_1_classifier.py)</t>
     </r>
   </si>
   <si>
@@ -33318,7 +33318,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Index examinations, n</t>
+      <t xml:space="preserve">S16 · Index examinations, n</t>
     </r>
   </si>
   <si>
@@ -33418,7 +33418,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Calendar days from index examination to operation, median (IQR)</t>
+      <t xml:space="preserve">S16 · Calendar days from index examination to operation, median (IQR)</t>
     </r>
   </si>
   <si>
@@ -33457,7 +33457,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Same day, n (%)</t>
+      <t xml:space="preserve">S16 · Same day, n (%)</t>
     </r>
   </si>
   <si>
@@ -33496,7 +33496,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · 1 day before, n (%)</t>
+      <t xml:space="preserve">S16 · 1 day before, n (%)</t>
     </r>
   </si>
   <si>
@@ -33535,7 +33535,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · 2–7 days before, n (%)</t>
+      <t xml:space="preserve">S16 · 2–7 days before, n (%)</t>
     </r>
   </si>
   <si>
@@ -33574,7 +33574,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · More than 7 days before, n (%)</t>
+      <t xml:space="preserve">S16 · More than 7 days before, n (%)</t>
     </r>
   </si>
   <si>
@@ -33613,7 +33613,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Detection, final label, closest episode (primary), n/N (%)</t>
+      <t xml:space="preserve">S16 · Detection, final label, closest episode (primary), n/N (%)</t>
     </r>
   </si>
   <si>
@@ -33652,7 +33652,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Detection, conclusion-only classifier, closest episode, n/N (%)</t>
+      <t xml:space="preserve">S16 · Detection, conclusion-only classifier, closest episode, n/N (%)</t>
     </r>
   </si>
   <si>
@@ -33691,7 +33691,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Detection, conclusion-only classifier, earliest episode, n/N (%)</t>
+      <t xml:space="preserve">S16 · Detection, conclusion-only classifier, earliest episode, n/N (%)</t>
     </r>
   </si>
   <si>
@@ -33730,7 +33730,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Detection, conclusion-only classifier, any preoperative episode positive, n/N (%)</t>
+      <t xml:space="preserve">S16 · Detection, conclusion-only classifier, any preoperative episode positive, n/N (%)</t>
     </r>
   </si>
   <si>
@@ -33769,7 +33769,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Children with more than one preoperative episode, n</t>
+      <t xml:space="preserve">S16 · Children with more than one preoperative episode, n</t>
     </r>
   </si>
   <si>
@@ -33808,7 +33808,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Detection, final label, examinations within 2 days of operation, n/N (%)</t>
+      <t xml:space="preserve">S16 · Detection, final label, examinations within 2 days of operation, n/N (%)</t>
     </r>
   </si>
   <si>
@@ -33847,7 +33847,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Adjusted OR vs UGI series, examinations within 2 days (95% CI)</t>
+      <t xml:space="preserve">S16 · Adjusted OR vs UGI series, examinations within 2 days (95% CI)</t>
     </r>
   </si>
   <si>
@@ -33886,7 +33886,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S18 · Adjusted OR vs CT, examinations within 2 days (95% CI)</t>
+      <t xml:space="preserve">S16 · Adjusted OR vs CT, examinations within 2 days (95% CI)</t>
     </r>
   </si>
   <si>
@@ -33925,7 +33925,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · All ultrasound examinations (primary denominator)</t>
+      <t xml:space="preserve">S17 · All ultrasound examinations (primary denominator)</t>
     </r>
   </si>
   <si>
@@ -34093,7 +34093,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · Booked as gastrointestinal</t>
+      <t xml:space="preserve">S17 · Booked as gastrointestinal</t>
     </r>
   </si>
   <si>
@@ -34261,7 +34261,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · Booked as abdominal great-vessel</t>
+      <t xml:space="preserve">S17 · Booked as abdominal great-vessel</t>
     </r>
   </si>
   <si>
@@ -34429,7 +34429,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · Booked as gastrointestinal or great-vessel</t>
+      <t xml:space="preserve">S17 · Booked as gastrointestinal or great-vessel</t>
     </r>
   </si>
   <si>
@@ -34597,7 +34597,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · Booked as pyloric only</t>
+      <t xml:space="preserve">S17 · Booked as pyloric only</t>
     </r>
   </si>
   <si>
@@ -34765,7 +34765,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · Performed at the bedside</t>
+      <t xml:space="preserve">S17 · Performed at the bedside</t>
     </r>
   </si>
   <si>
@@ -34933,7 +34933,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S19 · Child aged 28 days or younger</t>
+      <t xml:space="preserve">S17 · Child aged 28 days or younger</t>
     </r>
   </si>
   <si>
@@ -35340,7 +35340,7 @@
     <t xml:space="preserve">Title Page · Word count</t>
   </si>
   <si>
-    <t xml:space="preserve">2,976 … Abstract: 248 words</t>
+    <t xml:space="preserve">2,978 … Abstract: 248 words</t>
   </si>
   <si>
     <r>
@@ -35375,7 +35375,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2976</t>
+      <t xml:space="preserve">2978</t>
     </r>
     <r>
       <rPr>
@@ -35498,7 +35498,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Word count: 2,976 … Tables: 4; Figures: 3; Supplements 1–4</t>
+    <t xml:space="preserve">Word count: 2,978 … Tables: 4; Figures: 3; Supplements 1–4</t>
   </si>
   <si>
     <r>
@@ -35516,7 +35516,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2976</t>
+      <t xml:space="preserve">2978</t>
     </r>
   </si>
   <si>
@@ -38566,6 +38566,95 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">3 · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">正文（计数词）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> one</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">； </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">one in</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">； </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">three CT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Two features</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">补充</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">4 · A</t>
     </r>
     <r>
@@ -39545,7 +39634,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S8 </t>
+      <t xml:space="preserve">S18 </t>
     </r>
     <r>
       <rPr>
@@ -41386,7 +41475,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9</t>
+      <t xml:space="preserve">S8</t>
     </r>
   </si>
   <si>
@@ -42176,7 +42265,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S9</t>
+      <t xml:space="preserve">S8</t>
     </r>
     <r>
       <rPr>
@@ -43057,7 +43146,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S15 </t>
+      <t xml:space="preserve">S19 </t>
     </r>
     <r>
       <rPr>
@@ -43656,7 +43745,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2 · S2.7–S2.10 </t>
+      <t xml:space="preserve">2 · S2.7–S2.9 </t>
     </r>
     <r>
       <rPr>
@@ -43673,7 +43762,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">S16–S19</t>
+      <t xml:space="preserve">S14–S17</t>
     </r>
     <r>
       <rPr>
@@ -45158,7 +45247,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">COUNTA(核对表!B2:B2000)</f>
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45203,7 +45292,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTIF(核对表!C2:C2000,"【定义/描述性数字】*")</f>
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45231,7 +45320,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E355"/>
+  <dimension ref="A1:E356"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -49456,7 +49545,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="8" t="s">
         <v>683</v>
       </c>
@@ -51242,7 +51331,7 @@
       </c>
     </row>
     <row r="354" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A354" s="11" t="s">
+      <c r="A354" s="10" t="s">
         <v>944</v>
       </c>
       <c r="B354" s="11" t="s">
@@ -51275,8 +51364,25 @@
         <v>32</v>
       </c>
     </row>
+    <row r="356" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A356" s="11" t="s">
+        <v>948</v>
+      </c>
+      <c r="B356" s="11" t="s">
+        <v>949</v>
+      </c>
+      <c r="C356" s="10" t="s">
+        <v>893</v>
+      </c>
+      <c r="D356" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E356" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E355"/>
+  <autoFilter ref="A1:E356"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -51305,7 +51411,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>23</v>
@@ -51350,66 +51456,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>954</v>
+        <v>956</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>956</v>
+        <v>958</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>958</v>
+        <v>960</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>959</v>
+        <v>961</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>960</v>
+        <v>962</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>962</v>
+        <v>964</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>963</v>
+        <v>965</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>964</v>
+        <v>966</v>
       </c>
     </row>
   </sheetData>
@@ -51443,27 +51549,27 @@
         <v>23</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>966</v>
+        <v>968</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>967</v>
+        <v>969</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51471,13 +51577,13 @@
         <v>38</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>973</v>
+        <v>975</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>974</v>
+        <v>976</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51485,13 +51591,13 @@
         <v>134</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>977</v>
+        <v>979</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51499,13 +51605,13 @@
         <v>277</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>978</v>
+        <v>980</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>980</v>
+        <v>982</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51513,27 +51619,27 @@
         <v>283</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>981</v>
+        <v>983</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>984</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>982</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>980</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51541,27 +51647,27 @@
         <v>111</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>991</v>
+        <v>993</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>69</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51569,13 +51675,13 @@
         <v>127</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>994</v>
+        <v>996</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>995</v>
+        <v>997</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51583,13 +51689,13 @@
         <v>146</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>996</v>
+        <v>998</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51597,13 +51703,13 @@
         <v>368</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51611,13 +51717,13 @@
         <v>382</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51625,13 +51731,13 @@
         <v>385</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>1006</v>
+        <v>1008</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>1007</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51639,13 +51745,13 @@
         <v>397</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>1008</v>
+        <v>1010</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51653,265 +51759,265 @@
         <v>406</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>1011</v>
+        <v>1013</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>1016</v>
+        <v>1018</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>1018</v>
+        <v>1020</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1019</v>
+        <v>1021</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>1020</v>
+        <v>1022</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>1021</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>1023</v>
+        <v>1025</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>1024</v>
+        <v>1026</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>1025</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>1026</v>
+        <v>1028</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1027</v>
+        <v>1029</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>1028</v>
+        <v>1030</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>1029</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>1030</v>
+        <v>1032</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>1031</v>
+        <v>1033</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>1033</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>1034</v>
+        <v>1036</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>1046</v>
+        <v>1048</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>1047</v>
+        <v>1049</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>1048</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>1049</v>
+        <v>1051</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>1050</v>
+        <v>1052</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>1051</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>1052</v>
+        <v>1054</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>1053</v>
+        <v>1055</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>1054</v>
+        <v>1056</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>1055</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>1056</v>
+        <v>1058</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>1057</v>
+        <v>1059</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>1058</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>1059</v>
+        <v>1061</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>1060</v>
+        <v>1062</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>1061</v>
+        <v>1063</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>1062</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>1063</v>
+        <v>1065</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>1064</v>
+        <v>1066</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>1065</v>
+        <v>1067</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>1066</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>1067</v>
+        <v>1069</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>1068</v>
+        <v>1070</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>1069</v>
+        <v>1071</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>1070</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>1071</v>
+        <v>1073</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>1072</v>
+        <v>1074</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>1073</v>
+        <v>1075</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="69.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>1075</v>
+        <v>1077</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>1079</v>
+        <v>1081</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>1082</v>
+        <v>1084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Three wording fixes from the second pre-submission read
The abstract says excluding "possible" wording, matching Table 2. Supplement 1
no longer calls gastric volvulus benign. The Discussion says elements rather than
duodenal anatomy, since enteric fluid is listed too.

Main text 2,977 words; number check 355 rows, 0 inconsistent.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TkounLTBFVQRstE3VnhkM
</commit_message>
<xml_diff>
--- a/数字核对表.xlsx
+++ b/数字核对表.xlsx
@@ -35340,7 +35340,7 @@
     <t xml:space="preserve">Title Page · Word count</t>
   </si>
   <si>
-    <t xml:space="preserve">2,978 … Abstract: 248 words</t>
+    <t xml:space="preserve">2,977 … Abstract: 248 words</t>
   </si>
   <si>
     <r>
@@ -35375,7 +35375,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2978</t>
+      <t xml:space="preserve">2977</t>
     </r>
     <r>
       <rPr>
@@ -35498,7 +35498,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Word count: 2,978 … Tables: 4; Figures: 3; Supplements 1–4</t>
+    <t xml:space="preserve">Word count: 2,977 … Tables: 4; Figures: 3; Supplements 1–4</t>
   </si>
   <si>
     <r>
@@ -35516,7 +35516,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2978</t>
+      <t xml:space="preserve">2977</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
List ten authors: Guanghua Zhang, Hongxi Guo and Haibin Wang move from the acknowledgments to the author list
Title page, cover letter, CRediT statement, checks and operation sheet follow the
order agreed with the authors. EJR's guide sets no limit on the number of authors.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TkounLTBFVQRstE3VnhkM
</commit_message>
<xml_diff>
--- a/数字核对表.xlsx
+++ b/数字核对表.xlsx
@@ -35335,7 +35335,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">all seven authors</t>
+    <t xml:space="preserve">all ten authors</t>
   </si>
   <si>
     <r>
@@ -35370,7 +35370,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">7 </t>
+      <t xml:space="preserve">10 </t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
Supplement 1 in English only, as requested by the editorial office
All Chinese terms, example sentences and the content-audit patterns in Supplement 1
are replaced by English translations; Table S1 now gives the translated terms. The
original Chinese regular expressions and the database search strings are appended
to Supplement_1_classifier.py. New check: no Chinese characters in any uploaded file.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TkounLTBFVQRstE3VnhkM
</commit_message>
<xml_diff>
--- a/数字核对表.xlsx
+++ b/数字核对表.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">专项检查!$A$1:$B$8</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">更正记录!$A$1:$D$34</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$355</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">核对表!$A$1:$E$358</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">问题汇总!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1956" uniqueCount="1082">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1971" uniqueCount="1088">
   <si>
     <r>
       <rPr>
@@ -37828,6 +37828,80 @@
       </rPr>
       <t xml:space="preserve">by two independent</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">supp1.md:21</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（计数词）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">two written</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">supp1.md:35</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（计数词）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">two wordings</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">补充</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 · E1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（计数词）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> two Chinese</t>
   </si>
   <si>
     <r>
@@ -45137,7 +45211,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">COUNTA(核对表!B2:B2000)</f>
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45182,7 +45256,7 @@
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">COUNTIF(核对表!C2:C2000,"【定义/描述性数字】*")</f>
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45210,7 +45284,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E355"/>
+  <dimension ref="A1:E358"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -51051,7 +51125,7 @@
       </c>
     </row>
     <row r="344" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A344" s="10" t="s">
+      <c r="A344" s="11" t="s">
         <v>923</v>
       </c>
       <c r="B344" s="11" t="s">
@@ -51068,7 +51142,7 @@
       </c>
     </row>
     <row r="345" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A345" s="10" t="s">
+      <c r="A345" s="11" t="s">
         <v>925</v>
       </c>
       <c r="B345" s="11" t="s">
@@ -51221,7 +51295,7 @@
       </c>
     </row>
     <row r="354" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A354" s="11" t="s">
+      <c r="A354" s="10" t="s">
         <v>943</v>
       </c>
       <c r="B354" s="11" t="s">
@@ -51238,7 +51312,7 @@
       </c>
     </row>
     <row r="355" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A355" s="11" t="s">
+      <c r="A355" s="10" t="s">
         <v>945</v>
       </c>
       <c r="B355" s="11" t="s">
@@ -51254,8 +51328,59 @@
         <v>32</v>
       </c>
     </row>
+    <row r="356" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A356" s="10" t="s">
+        <v>947</v>
+      </c>
+      <c r="B356" s="11" t="s">
+        <v>948</v>
+      </c>
+      <c r="C356" s="10" t="s">
+        <v>892</v>
+      </c>
+      <c r="D356" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E356" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="357" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A357" s="11" t="s">
+        <v>949</v>
+      </c>
+      <c r="B357" s="11" t="s">
+        <v>950</v>
+      </c>
+      <c r="C357" s="10" t="s">
+        <v>892</v>
+      </c>
+      <c r="D357" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E357" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="358" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A358" s="11" t="s">
+        <v>951</v>
+      </c>
+      <c r="B358" s="11" t="s">
+        <v>952</v>
+      </c>
+      <c r="C358" s="10" t="s">
+        <v>892</v>
+      </c>
+      <c r="D358" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E358" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E355"/>
+  <autoFilter ref="A1:E358"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -51284,7 +51409,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>23</v>
@@ -51329,66 +51454,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
     </row>
   </sheetData>
@@ -51422,27 +51547,27 @@
         <v>23</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51450,13 +51575,13 @@
         <v>38</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51464,13 +51589,13 @@
         <v>134</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51478,13 +51603,13 @@
         <v>282</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51492,27 +51617,27 @@
         <v>288</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51520,27 +51645,27 @@
         <v>111</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>988</v>
+        <v>994</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>989</v>
+        <v>995</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>69</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51548,13 +51673,13 @@
         <v>127</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>992</v>
+        <v>998</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51562,13 +51687,13 @@
         <v>146</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>995</v>
+        <v>1001</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>997</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51576,13 +51701,13 @@
         <v>373</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>998</v>
+        <v>1004</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>999</v>
+        <v>1005</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51590,13 +51715,13 @@
         <v>387</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>1002</v>
+        <v>1008</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>1003</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51604,13 +51729,13 @@
         <v>390</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>1005</v>
+        <v>1011</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>1006</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51618,13 +51743,13 @@
         <v>402</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>1007</v>
+        <v>1013</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>1008</v>
+        <v>1014</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>1009</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51632,265 +51757,265 @@
         <v>411</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>1011</v>
+        <v>1017</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>1012</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>1013</v>
+        <v>1019</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>1014</v>
+        <v>1020</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>1015</v>
+        <v>1021</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>1016</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>1017</v>
+        <v>1023</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1018</v>
+        <v>1024</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>1019</v>
+        <v>1025</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>1020</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>1021</v>
+        <v>1027</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>1022</v>
+        <v>1028</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>1023</v>
+        <v>1029</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>1024</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>1025</v>
+        <v>1031</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1026</v>
+        <v>1032</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>1029</v>
+        <v>1035</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>1030</v>
+        <v>1036</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>1031</v>
+        <v>1037</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>1032</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>1033</v>
+        <v>1039</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1034</v>
+        <v>1040</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>1035</v>
+        <v>1041</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>1036</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>1038</v>
+        <v>1044</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>1039</v>
+        <v>1045</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>1041</v>
+        <v>1047</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>1043</v>
+        <v>1049</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>1035</v>
+        <v>1041</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>1047</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>1049</v>
+        <v>1055</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>1050</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>1053</v>
+        <v>1059</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>1054</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>100</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>1061</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>1062</v>
+        <v>1068</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>1063</v>
+        <v>1069</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>1064</v>
+        <v>1070</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>1065</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="58.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>1066</v>
+        <v>1072</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>1067</v>
+        <v>1073</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>1070</v>
+        <v>1076</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>1071</v>
+        <v>1077</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>1073</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="69.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>1075</v>
+        <v>1081</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>1076</v>
+        <v>1082</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>1077</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>1078</v>
+        <v>1084</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>1079</v>
+        <v>1085</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>1080</v>
+        <v>1086</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>1081</v>
+        <v>1087</v>
       </c>
     </row>
   </sheetData>

</xml_diff>